<commit_message>
Use valid IEK catalog SKUs in invoice fixture
</commit_message>
<xml_diff>
--- a/fixtures/documents/iek_invoice_demo.xlsx
+++ b/fixtures/documents/iek_invoice_demo.xlsx
@@ -453,13 +453,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>0</v>
+        <v>010300001_</v>
       </c>
       <c r="B7" t="str">
-        <v>Расширение 3кв 24</v>
+        <v>MAD10-2-010-C-030</v>
       </c>
       <c r="C7" t="str">
-        <v>0</v>
+        <v>УЗО АД 12  (2ф) 10А IEK (5/40)</v>
       </c>
       <c r="D7">
         <v>60</v>
@@ -476,13 +476,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>010300001_</v>
+        <v>010300002_</v>
       </c>
       <c r="B8" t="str">
-        <v>MAD10-2-010-C-030</v>
+        <v>MAD10-2-016-C-030</v>
       </c>
       <c r="C8" t="str">
-        <v>УЗО АД 12  (2ф) 10А IEK (5/40)</v>
+        <v>УЗО АД 12  (2ф) 16А IEK (5/40)</v>
       </c>
       <c r="D8">
         <v>20</v>
@@ -499,13 +499,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>010300002_</v>
+        <v>010300003_</v>
       </c>
       <c r="B9" t="str">
-        <v>MAD10-2-016-C-030</v>
+        <v>MAD10-2-025-C-030</v>
       </c>
       <c r="C9" t="str">
-        <v>УЗО АД 12  (2ф) 16А IEK (5/40)</v>
+        <v>УЗО АД 12  (2ф) 25А IEK (5/40)</v>
       </c>
       <c r="D9">
         <v>20</v>
@@ -522,13 +522,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>010300003_</v>
+        <v>010300004_</v>
       </c>
       <c r="B10" t="str">
-        <v>MAD10-2-025-C-030</v>
+        <v>MAD10-2-032-C-030</v>
       </c>
       <c r="C10" t="str">
-        <v>УЗО АД 12  (2ф) 25А IEK (5/40)</v>
+        <v>УЗО АД 12  (2ф) 32А IEK (5/40)</v>
       </c>
       <c r="D10">
         <v>20</v>
@@ -545,13 +545,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>010300004_</v>
+        <v>010300005_</v>
       </c>
       <c r="B11" t="str">
-        <v>MAD10-2-032-C-030</v>
+        <v>MAD10-2-040-C-030</v>
       </c>
       <c r="C11" t="str">
-        <v>УЗО АД 12  (2ф) 32А IEK (5/40)</v>
+        <v>УЗО АД 12  (2ф) 40А IEK (4/32)</v>
       </c>
       <c r="D11">
         <v>20</v>
@@ -568,13 +568,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>010300005_</v>
+        <v>010300006_</v>
       </c>
       <c r="B12" t="str">
-        <v>MAD10-2-040-C-030</v>
+        <v>MAD10-2-050-C-030</v>
       </c>
       <c r="C12" t="str">
-        <v>УЗО АД 12  (2ф) 40А IEK (4/32)</v>
+        <v>УЗО АД 12  (2ф) 50А IEK (4/32)</v>
       </c>
       <c r="D12">
         <v>20</v>
@@ -591,13 +591,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>010300006_</v>
+        <v>010300007_</v>
       </c>
       <c r="B13" t="str">
-        <v>MAD10-2-050-C-030</v>
+        <v>MAD10-2-063-C-030</v>
       </c>
       <c r="C13" t="str">
-        <v>УЗО АД 12  (2ф) 50А IEK (4/32)</v>
+        <v>УЗО АД 12  (2ф) 63А IEK (4/32)</v>
       </c>
       <c r="D13">
         <v>20</v>
@@ -614,13 +614,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>010300007_</v>
+        <v>010300008_</v>
       </c>
       <c r="B14" t="str">
-        <v>MAD10-2-063-C-030</v>
+        <v>MAD10-4-016-C-030</v>
       </c>
       <c r="C14" t="str">
-        <v>УЗО АД 12  (2ф) 63А IEK (4/32)</v>
+        <v>УЗО АД 14  (4ф) 16А IEK (3/24)</v>
       </c>
       <c r="D14">
         <v>20</v>
@@ -637,13 +637,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>010300008_</v>
+        <v>010300009_</v>
       </c>
       <c r="B15" t="str">
-        <v>MAD10-4-016-C-030</v>
+        <v>MAD10-4-025-C-030</v>
       </c>
       <c r="C15" t="str">
-        <v>УЗО АД 14  (4ф) 16А IEK (3/24)</v>
+        <v>УЗО АД 14  (4ф) 25А IEK (3/24)</v>
       </c>
       <c r="D15">
         <v>20</v>
@@ -660,13 +660,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>010300009_</v>
+        <v>010300010_</v>
       </c>
       <c r="B16" t="str">
-        <v>MAD10-4-025-C-030</v>
+        <v>MAD10-4-032-C-030</v>
       </c>
       <c r="C16" t="str">
-        <v>УЗО АД 14  (4ф) 25А IEK (3/24)</v>
+        <v>УЗО АД 14  (4ф) 32А IEK (3/24)</v>
       </c>
       <c r="D16">
         <v>20</v>

</xml_diff>